<commit_message>
update: plantilla para importar alumnos
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/Plantilla Importar Alumnos.xlsx
+++ b/src/main/resources/templates/Plantilla Importar Alumnos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anton\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8AC8D1A-6D48-4BA2-A424-6FA88B501B01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ACBB149-44CE-46B3-B7D1-62737046CB84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{377B9857-FFD6-4EAF-8EF7-352E7BF8EAF3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{377B9857-FFD6-4EAF-8EF7-352E7BF8EAF3}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="3" r:id="rId1"/>
@@ -40,23 +40,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
   <si>
     <t>DNI</t>
   </si>
   <si>
-    <t>NOMBRE</t>
-  </si>
-  <si>
     <t>AREA</t>
   </si>
   <si>
     <t>TUTOR</t>
   </si>
   <si>
-    <t>ACOSTA CHAVELON XIARA</t>
-  </si>
-  <si>
     <t>Letras</t>
   </si>
   <si>
@@ -88,13 +82,31 @@
   </si>
   <si>
     <t>Silvia</t>
+  </si>
+  <si>
+    <t>APELLIDO PATERNO</t>
+  </si>
+  <si>
+    <t>APELLIDO MATERNO</t>
+  </si>
+  <si>
+    <t>NOMBRES</t>
+  </si>
+  <si>
+    <t>ACOSTA</t>
+  </si>
+  <si>
+    <t>CHAVELÓN</t>
+  </si>
+  <si>
+    <t>XIARA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -103,36 +115,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="1"/>
-      <name val="Teko"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Gill Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Libre Franklin"/>
     </font>
   </fonts>
   <fills count="4">
@@ -182,26 +167,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -543,86 +513,114 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76E12E3D-48CC-4488-B9D0-215D855C9C11}">
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.5546875" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" customWidth="1"/>
-    <col min="4" max="4" width="22.21875" customWidth="1"/>
+    <col min="1" max="3" width="22.5546875" customWidth="1"/>
+    <col min="4" max="4" width="30.88671875" customWidth="1"/>
+    <col min="5" max="5" width="18.6640625" customWidth="1"/>
+    <col min="6" max="6" width="22.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="22.8">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3" t="s">
+    </row>
+    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>78456321</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="22.8">
+      <c r="F2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="4"/>
-    </row>
-    <row r="4" spans="1:4" ht="22.8">
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4" ht="22.8">
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4" ht="22.8">
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="1:4" ht="22.8">
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4" ht="22.8">
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="6"/>
-    </row>
-    <row r="9" spans="1:4" ht="22.8">
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="7"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D8" xr:uid="{02A3D613-1A7F-47BC-8CC1-AB80325B7B71}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F8" xr:uid="{02A3D613-1A7F-47BC-8CC1-AB80325B7B71}">
       <formula1>"CLAUDIA,PAUL"</formula1>
     </dataValidation>
   </dataValidations>
@@ -633,7 +631,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{970AAC77-C7A2-4419-A9A2-79115A387D55}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.5546875" customWidth="1"/>
     <col min="4" max="4" width="33.77734375" customWidth="1"/>
@@ -642,54 +640,54 @@
     <col min="8" max="8" width="54.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="42" customHeight="1">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="H1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="8"/>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" t="s">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>